<commit_message>
Parche de errores Backend - bugs front-end
</commit_message>
<xml_diff>
--- a/Backend/src/modules/importaciones/plantillas/motorizados.xlsx
+++ b/Backend/src/modules/importaciones/plantillas/motorizados.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="22">
   <si>
     <t>usuario</t>
   </si>
@@ -20,9 +20,6 @@
     <t>placa</t>
   </si>
   <si>
-    <t>estado</t>
-  </si>
-  <si>
     <t>Instrucciones — Plantilla de Motorizados</t>
   </si>
   <si>
@@ -69,9 +66,6 @@
   </si>
   <si>
     <t>Placa del vehiculo.</t>
-  </si>
-  <si>
-    <t>Estado del motorizado (ej. disponible, en_ruta — igual al enum ya usado por el sistema).</t>
   </si>
   <si>
     <t>Duplicados</t>
@@ -497,21 +491,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C1"/>
+  <dimension ref="A1:B1"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="3" width="14" customWidth="1"/>
+    <col min="1" max="2" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="20" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -522,7 +513,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B1:D22"/>
+  <dimension ref="B1:D21"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="4" customWidth="1"/>
@@ -533,63 +524,63 @@
   <sheetData>
     <row r="1" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B1" s="2" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B3" s="3" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="5" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="6" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="7" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B7" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="8" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="9" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="10" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="12" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B12" s="3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="13" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B13" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C13" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="C13" s="1" t="s">
+      <c r="D13" s="1" t="s">
         <v>14</v>
-      </c>
-      <c r="D13" s="1" t="s">
-        <v>15</v>
       </c>
     </row>
     <row r="14" spans="2:4" x14ac:dyDescent="0.25">
@@ -597,10 +588,10 @@
         <v>0</v>
       </c>
       <c r="C14" t="s">
+        <v>15</v>
+      </c>
+      <c r="D14" t="s">
         <v>16</v>
-      </c>
-      <c r="D14" t="s">
-        <v>17</v>
       </c>
     </row>
     <row r="15" spans="2:4" x14ac:dyDescent="0.25">
@@ -608,41 +599,30 @@
         <v>1</v>
       </c>
       <c r="C15" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D15" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="17" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B17" s="3" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="16" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B16" t="s">
-        <v>2</v>
-      </c>
-      <c r="C16" t="s">
-        <v>16</v>
-      </c>
-      <c r="D16" t="s">
+    <row r="18" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B18" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="18" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B18" s="3" t="s">
+    <row r="20" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B20" s="3" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="19" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B19" t="s">
+    <row r="21" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B21" t="s">
         <v>21</v>
-      </c>
-    </row>
-    <row r="21" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B21" s="3" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="22" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B22" t="s">
-        <v>23</v>
       </c>
     </row>
   </sheetData>

</xml_diff>